<commit_message>
add baton id support
</commit_message>
<xml_diff>
--- a/templates/baton-file-excel-template.xlsx
+++ b/templates/baton-file-excel-template.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Quickstart" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Instructions" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Users" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Resources" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Entitlements" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="Direct User Grants" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="Grant Inheritance Mappings" sheetId="7" r:id="rId11"/>
+    <sheet name="Quickstart" sheetId="1" r:id="rId5" state="visible"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId6" state="visible"/>
+    <sheet name="Users" sheetId="3" r:id="rId7" state="visible"/>
+    <sheet name="Resources" sheetId="4" r:id="rId8" state="visible"/>
+    <sheet name="Entitlements" sheetId="5" r:id="rId9" state="visible"/>
+    <sheet name="Direct User Grants" sheetId="6" r:id="rId10" state="visible"/>
+    <sheet name="Grant Inheritance Mappings" sheetId="7" r:id="rId11" state="visible"/>
+    <sheet name="External Grants" sheetId="8" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -17,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="294">
   <si>
     <t>QUICKSTART GUIDE</t>
   </si>
@@ -803,22 +804,118 @@
   </si>
   <si>
     <t>shallow</t>
+  </si>
+  <si>
+    <t>Match Type</t>
+  </si>
+  <si>
+    <t>Match Resource Type</t>
+  </si>
+  <si>
+    <t>Match ID</t>
+  </si>
+  <si>
+    <t>Match Key</t>
+  </si>
+  <si>
+    <t>Match Value</t>
+  </si>
+  <si>
+    <t>attribute</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>jane.smith@external.com</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>external-group-123</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>This workbook defines identity and access data for the ConductorOne Baton file connector. The connector reads data from sheets named 'Users', 'Resources', 'Entitlements', 'Direct User Grants', 'Grant Inheritance Mappings', and 'External Grants'. Column order does not matter, but header names in Row 1 must match exactly (case-insensitive). This 'Instructions' sheet is ignored by the connector.</t>
+  </si>
+  <si>
+    <t>Sheet: External Grants</t>
+  </si>
+  <si>
+    <t>Defines grants to principals owned by ANOTHER connector (the 'shared identity source', e.g. Okta or Active Directory). The principal is NOT defined in this workbook — a match rule tells ConductorOne how to find it in the identity source's data. Requires configuring a shared identity source for this connector in ConductorOne.</t>
+  </si>
+  <si>
+    <t>External Grants</t>
+  </si>
+  <si>
+    <t>The ID of the local resource that owns the entitlement being granted. Must match a Resource ID in 'Entitlements'.</t>
+  </si>
+  <si>
+    <t>How to find the external principal. 'all' = every external principal of the given type. 'id' = match one principal by its native ID. 'attribute' = match by an attribute key/value pair.</t>
+  </si>
+  <si>
+    <t>all, id, attribute</t>
+  </si>
+  <si>
+    <t>The external principal's type. Valid values: user, group.</t>
+  </si>
+  <si>
+    <t>user, group</t>
+  </si>
+  <si>
+    <t>If Match Type = id</t>
+  </si>
+  <si>
+    <t>The external principal's native ID in the identity source.</t>
+  </si>
+  <si>
+    <t>If Match Type = attribute</t>
+  </si>
+  <si>
+    <t>The attribute to match on. 'email' is the standard supported key for users.</t>
+  </si>
+  <si>
+    <t>The attribute value to match.</t>
+  </si>
+  <si>
+    <t>8. External Grants reference the Entitlements sheet the same way Direct User Grants do. The Match columns describe principals in the shared identity source, NOT in this workbook.</t>
+  </si>
+  <si>
+    <t>Expand Entitlement Slug</t>
+  </si>
+  <si>
+    <t>Expand Depth</t>
+  </si>
+  <si>
+    <t>Optional grant expansion: members of the matched external group inherit this grant through the group's named entitlement. Only valid when Match Resource Type is 'group' and Match Type is 'id' or 'attribute'.</t>
+  </si>
+  <si>
+    <t>How deep the expansion goes. 'full' = transitive (default). 'shallow' = one level only. Only meaningful when Expand Entitlement Slug is set.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <fonts count="2">
     <font>
-      <sz val="10.0"/>
+      <name val="Arial"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <color theme="1"/>
-      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -834,21 +931,21 @@
     <border/>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyAlignment="true"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
     </xf>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyFont="true" applyAlignment="true">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
 </styleSheet>
@@ -859,7 +956,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1077,15 +1174,17 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -1426,9 +1525,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -1437,7 +1536,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4">
@@ -2203,213 +2302,391 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="s">
-        <v>175</v>
+      <c r="A55" t="s">
+        <v>276</v>
+      </c>
+      <c r="B55" t="s">
+        <v>277</v>
+      </c>
+      <c r="C55" t="s">
+        <v>269</v>
+      </c>
+      <c r="D55" t="s">
+        <v>269</v>
+      </c>
+      <c r="E55" t="s">
+        <v>269</v>
+      </c>
+      <c r="F55" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="s">
-        <v>176</v>
+      <c r="A56" t="s">
+        <v>278</v>
+      </c>
+      <c r="B56" t="s">
+        <v>40</v>
+      </c>
+      <c r="C56" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" t="s">
+        <v>279</v>
+      </c>
+      <c r="E56" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>6</v>
+      <c r="A57" t="s">
+        <v>278</v>
+      </c>
+      <c r="B57" t="s">
+        <v>41</v>
+      </c>
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
+        <v>155</v>
+      </c>
+      <c r="E57" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>75</v>
+      <c r="A58" t="s">
+        <v>278</v>
+      </c>
+      <c r="B58" t="s">
+        <v>262</v>
+      </c>
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>180</v>
+      <c r="A59" t="s">
+        <v>278</v>
+      </c>
+      <c r="B59" t="s">
+        <v>263</v>
+      </c>
+      <c r="C59" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" t="s">
+        <v>282</v>
+      </c>
+      <c r="E59" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>182</v>
+      <c r="A60" t="s">
+        <v>278</v>
+      </c>
+      <c r="B60" t="s">
+        <v>264</v>
+      </c>
+      <c r="C60" t="s">
+        <v>284</v>
+      </c>
+      <c r="D60" t="s">
+        <v>285</v>
+      </c>
+      <c r="E60" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>184</v>
+      <c r="A61" t="s">
+        <v>278</v>
+      </c>
+      <c r="B61" t="s">
+        <v>265</v>
+      </c>
+      <c r="C61" t="s">
+        <v>286</v>
+      </c>
+      <c r="D61" t="s">
+        <v>287</v>
+      </c>
+      <c r="E61" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>186</v>
+      <c r="A62" t="s">
+        <v>278</v>
+      </c>
+      <c r="B62" t="s">
+        <v>266</v>
+      </c>
+      <c r="C62" t="s">
+        <v>286</v>
+      </c>
+      <c r="D62" t="s">
+        <v>288</v>
+      </c>
+      <c r="E62" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="s">
-        <v>189</v>
+      <c r="A63" t="s">
+        <v>278</v>
+      </c>
+      <c r="B63" t="s">
+        <v>290</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>292</v>
+      </c>
+      <c r="E63" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>278</v>
+      </c>
+      <c r="B64" t="s">
+        <v>291</v>
+      </c>
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>293</v>
+      </c>
+      <c r="E64" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="s">
-        <v>192</v>
+        <v>177</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="s">
-        <v>193</v>
+        <v>178</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="s">
-        <v>194</v>
+        <v>179</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="s">
-        <v>195</v>
+        <v>181</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="s">
-        <v>196</v>
+        <v>183</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="1" t="s">
-        <v>198</v>
+        <v>187</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G77" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G80" s="1" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B94" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C82" s="1" t="s">
+      <c r="C94" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="G82" s="1" t="s">
+      <c r="G94" s="1" t="s">
         <v>207</v>
       </c>
     </row>
@@ -2421,9 +2698,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2567,9 +2844,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2735,9 +3012,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2817,9 +3094,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2884,9 +3161,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2942,4 +3219,119 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="9" min="1" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D2" t="s">
+        <v>268</v>
+      </c>
+      <c r="E2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" t="s">
+        <v>273</v>
+      </c>
+      <c r="F3" t="s">
+        <v>269</v>
+      </c>
+      <c r="G3" t="s">
+        <v>269</v>
+      </c>
+      <c r="H3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C4" t="s">
+        <v>274</v>
+      </c>
+      <c r="D4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G4" t="s">
+        <v>269</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add baton id support (#46)
* add baton id support

* lint: replace repeated string literals with constants in client package

goconst counts occurrences in _test.go files toward its threshold even
though reports there are excluded, so the "full" and "group" literals in
loader.go tripped the linter once the external-grant tests landed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/baton-file-excel-template.xlsx
+++ b/templates/baton-file-excel-template.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Quickstart" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Instructions" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Users" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Resources" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Entitlements" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="Direct User Grants" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="Grant Inheritance Mappings" sheetId="7" r:id="rId11"/>
+    <sheet name="Quickstart" sheetId="1" r:id="rId5" state="visible"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId6" state="visible"/>
+    <sheet name="Users" sheetId="3" r:id="rId7" state="visible"/>
+    <sheet name="Resources" sheetId="4" r:id="rId8" state="visible"/>
+    <sheet name="Entitlements" sheetId="5" r:id="rId9" state="visible"/>
+    <sheet name="Direct User Grants" sheetId="6" r:id="rId10" state="visible"/>
+    <sheet name="Grant Inheritance Mappings" sheetId="7" r:id="rId11" state="visible"/>
+    <sheet name="External Grants" sheetId="8" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -17,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="294">
   <si>
     <t>QUICKSTART GUIDE</t>
   </si>
@@ -803,22 +804,118 @@
   </si>
   <si>
     <t>shallow</t>
+  </si>
+  <si>
+    <t>Match Type</t>
+  </si>
+  <si>
+    <t>Match Resource Type</t>
+  </si>
+  <si>
+    <t>Match ID</t>
+  </si>
+  <si>
+    <t>Match Key</t>
+  </si>
+  <si>
+    <t>Match Value</t>
+  </si>
+  <si>
+    <t>attribute</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>jane.smith@external.com</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>external-group-123</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>This workbook defines identity and access data for the ConductorOne Baton file connector. The connector reads data from sheets named 'Users', 'Resources', 'Entitlements', 'Direct User Grants', 'Grant Inheritance Mappings', and 'External Grants'. Column order does not matter, but header names in Row 1 must match exactly (case-insensitive). This 'Instructions' sheet is ignored by the connector.</t>
+  </si>
+  <si>
+    <t>Sheet: External Grants</t>
+  </si>
+  <si>
+    <t>Defines grants to principals owned by ANOTHER connector (the 'shared identity source', e.g. Okta or Active Directory). The principal is NOT defined in this workbook — a match rule tells ConductorOne how to find it in the identity source's data. Requires configuring a shared identity source for this connector in ConductorOne.</t>
+  </si>
+  <si>
+    <t>External Grants</t>
+  </si>
+  <si>
+    <t>The ID of the local resource that owns the entitlement being granted. Must match a Resource ID in 'Entitlements'.</t>
+  </si>
+  <si>
+    <t>How to find the external principal. 'all' = every external principal of the given type. 'id' = match one principal by its native ID. 'attribute' = match by an attribute key/value pair.</t>
+  </si>
+  <si>
+    <t>all, id, attribute</t>
+  </si>
+  <si>
+    <t>The external principal's type. Valid values: user, group.</t>
+  </si>
+  <si>
+    <t>user, group</t>
+  </si>
+  <si>
+    <t>If Match Type = id</t>
+  </si>
+  <si>
+    <t>The external principal's native ID in the identity source.</t>
+  </si>
+  <si>
+    <t>If Match Type = attribute</t>
+  </si>
+  <si>
+    <t>The attribute to match on. 'email' is the standard supported key for users.</t>
+  </si>
+  <si>
+    <t>The attribute value to match.</t>
+  </si>
+  <si>
+    <t>8. External Grants reference the Entitlements sheet the same way Direct User Grants do. The Match columns describe principals in the shared identity source, NOT in this workbook.</t>
+  </si>
+  <si>
+    <t>Expand Entitlement Slug</t>
+  </si>
+  <si>
+    <t>Expand Depth</t>
+  </si>
+  <si>
+    <t>Optional grant expansion: members of the matched external group inherit this grant through the group's named entitlement. Only valid when Match Resource Type is 'group' and Match Type is 'id' or 'attribute'.</t>
+  </si>
+  <si>
+    <t>How deep the expansion goes. 'full' = transitive (default). 'shallow' = one level only. Only meaningful when Expand Entitlement Slug is set.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <fonts count="2">
     <font>
-      <sz val="10.0"/>
+      <name val="Arial"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <color theme="1"/>
-      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -834,21 +931,21 @@
     <border/>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyAlignment="true"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
+      <alignment/>
     </xf>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyFont="true" applyAlignment="true">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
 </styleSheet>
@@ -859,7 +956,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1077,15 +1174,17 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -1426,9 +1525,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -1437,7 +1536,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4">
@@ -2203,213 +2302,391 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="s">
-        <v>175</v>
+      <c r="A55" t="s">
+        <v>276</v>
+      </c>
+      <c r="B55" t="s">
+        <v>277</v>
+      </c>
+      <c r="C55" t="s">
+        <v>269</v>
+      </c>
+      <c r="D55" t="s">
+        <v>269</v>
+      </c>
+      <c r="E55" t="s">
+        <v>269</v>
+      </c>
+      <c r="F55" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="s">
-        <v>176</v>
+      <c r="A56" t="s">
+        <v>278</v>
+      </c>
+      <c r="B56" t="s">
+        <v>40</v>
+      </c>
+      <c r="C56" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" t="s">
+        <v>279</v>
+      </c>
+      <c r="E56" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>6</v>
+      <c r="A57" t="s">
+        <v>278</v>
+      </c>
+      <c r="B57" t="s">
+        <v>41</v>
+      </c>
+      <c r="C57" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" t="s">
+        <v>155</v>
+      </c>
+      <c r="E57" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>75</v>
+      <c r="A58" t="s">
+        <v>278</v>
+      </c>
+      <c r="B58" t="s">
+        <v>262</v>
+      </c>
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" t="s">
+        <v>280</v>
+      </c>
+      <c r="E58" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>180</v>
+      <c r="A59" t="s">
+        <v>278</v>
+      </c>
+      <c r="B59" t="s">
+        <v>263</v>
+      </c>
+      <c r="C59" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" t="s">
+        <v>282</v>
+      </c>
+      <c r="E59" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>182</v>
+      <c r="A60" t="s">
+        <v>278</v>
+      </c>
+      <c r="B60" t="s">
+        <v>264</v>
+      </c>
+      <c r="C60" t="s">
+        <v>284</v>
+      </c>
+      <c r="D60" t="s">
+        <v>285</v>
+      </c>
+      <c r="E60" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>184</v>
+      <c r="A61" t="s">
+        <v>278</v>
+      </c>
+      <c r="B61" t="s">
+        <v>265</v>
+      </c>
+      <c r="C61" t="s">
+        <v>286</v>
+      </c>
+      <c r="D61" t="s">
+        <v>287</v>
+      </c>
+      <c r="E61" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>186</v>
+      <c r="A62" t="s">
+        <v>278</v>
+      </c>
+      <c r="B62" t="s">
+        <v>266</v>
+      </c>
+      <c r="C62" t="s">
+        <v>286</v>
+      </c>
+      <c r="D62" t="s">
+        <v>288</v>
+      </c>
+      <c r="E62" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="s">
-        <v>189</v>
+      <c r="A63" t="s">
+        <v>278</v>
+      </c>
+      <c r="B63" t="s">
+        <v>290</v>
+      </c>
+      <c r="C63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D63" t="s">
+        <v>292</v>
+      </c>
+      <c r="E63" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>278</v>
+      </c>
+      <c r="B64" t="s">
+        <v>291</v>
+      </c>
+      <c r="C64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D64" t="s">
+        <v>293</v>
+      </c>
+      <c r="E64" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="s">
-        <v>192</v>
+        <v>177</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="s">
-        <v>193</v>
+        <v>178</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="s">
-        <v>194</v>
+        <v>179</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="s">
-        <v>195</v>
+        <v>181</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="s">
-        <v>196</v>
+        <v>183</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="1" t="s">
-        <v>198</v>
+        <v>187</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G77" s="1" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G80" s="1" t="s">
-        <v>207</v>
+        <v>193</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="B94" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C82" s="1" t="s">
+      <c r="C94" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="G82" s="1" t="s">
+      <c r="G94" s="1" t="s">
         <v>207</v>
       </c>
     </row>
@@ -2421,9 +2698,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2567,9 +2844,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2735,9 +3012,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2817,9 +3094,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2884,9 +3161,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryBelow="false" summaryRight="false"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="true"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -2942,4 +3219,119 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="9" min="1" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D2" t="s">
+        <v>268</v>
+      </c>
+      <c r="E2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" t="s">
+        <v>273</v>
+      </c>
+      <c r="F3" t="s">
+        <v>269</v>
+      </c>
+      <c r="G3" t="s">
+        <v>269</v>
+      </c>
+      <c r="H3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C4" t="s">
+        <v>274</v>
+      </c>
+      <c r="D4" t="s">
+        <v>268</v>
+      </c>
+      <c r="E4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G4" t="s">
+        <v>269</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>